<commit_message>
finished circuits of both hospital rover and product display with speakers and steppers projects
</commit_message>
<xml_diff>
--- a/product_display_stepper_speaker/BOM.xlsx
+++ b/product_display_stepper_speaker/BOM.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="38">
   <si>
     <t xml:space="preserve">No.</t>
   </si>
@@ -43,22 +43,97 @@
     <t xml:space="preserve">Store</t>
   </si>
   <si>
-    <t xml:space="preserve">Raspberry Pi Pico W</t>
+    <t xml:space="preserve">ESP-12E</t>
   </si>
   <si>
     <t xml:space="preserve">soldered</t>
   </si>
   <si>
+    <t xml:space="preserve">Male 2mm 1x8 Header</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Female 2mm 1x8 Header</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Female 2.54mm 1x3 Header</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Male 2.54mm 1x2 Header</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Male 2.54mm 1x11 Header</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Approx</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Push Button</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Given</t>
+  </si>
+  <si>
+    <t xml:space="preserve">JST Male 2Pin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">JST Female 2Pin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">JST Female 4Pin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">JST 4p to stepper cable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DRV8825</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PAM8403</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Speaker 3W</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nema17 25mm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Resistors</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Capacitors</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LD33v</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L7805</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Barrel Jack Female</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Barrel Jack Male wire</t>
+  </si>
+  <si>
+    <t xml:space="preserve">18650 li-ion</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BMS 3s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nickel Strips</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PCB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Delivery</t>
+  </si>
+  <si>
     <t xml:space="preserve">Development, manufacturing testing</t>
   </si>
   <si>
     <t xml:space="preserve">TOTAL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Approx</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Given</t>
   </si>
 </sst>
 </file>
@@ -478,8 +553,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G1048576"/>
-  <sheetFormatPr defaultColWidth="10.53125" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:J36"/>
+  <sheetFormatPr defaultColWidth="10.5390625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="4"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="31.39"/>
@@ -521,15 +596,13 @@
       <c r="B2" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="7" t="n">
-        <v>650</v>
-      </c>
+      <c r="C2" s="7"/>
       <c r="D2" s="7" t="n">
         <v>1</v>
       </c>
       <c r="E2" s="8" t="n">
         <f aca="false">C2*D2</f>
-        <v>650</v>
+        <v>0</v>
       </c>
       <c r="F2" s="9" t="s">
         <v>8</v>
@@ -540,9 +613,13 @@
       <c r="A3" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="11"/>
+      <c r="B3" s="11" t="s">
+        <v>9</v>
+      </c>
       <c r="C3" s="12"/>
-      <c r="D3" s="12"/>
+      <c r="D3" s="12" t="n">
+        <v>2</v>
+      </c>
       <c r="E3" s="13" t="n">
         <f aca="false">C3*D3</f>
         <v>0</v>
@@ -554,9 +631,13 @@
       <c r="A4" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="11"/>
+      <c r="B4" s="11" t="s">
+        <v>10</v>
+      </c>
       <c r="C4" s="12"/>
-      <c r="D4" s="12"/>
+      <c r="D4" s="12" t="n">
+        <v>2</v>
+      </c>
       <c r="E4" s="13" t="n">
         <f aca="false">C4*D4</f>
         <v>0</v>
@@ -568,13 +649,14 @@
       <c r="A5" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="11"/>
+      <c r="B5" s="11" t="s">
+        <v>11</v>
+      </c>
       <c r="C5" s="12"/>
-      <c r="D5" s="12"/>
-      <c r="E5" s="13" t="n">
-        <f aca="false">C5*D5</f>
-        <v>0</v>
-      </c>
+      <c r="D5" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" s="13"/>
       <c r="F5" s="14"/>
       <c r="G5" s="13"/>
     </row>
@@ -582,94 +664,397 @@
       <c r="A6" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="11"/>
+      <c r="B6" s="11" t="s">
+        <v>12</v>
+      </c>
       <c r="C6" s="12"/>
-      <c r="D6" s="12"/>
-      <c r="E6" s="13" t="n">
-        <f aca="false">C6*D6</f>
-        <v>0</v>
-      </c>
+      <c r="D6" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" s="13"/>
+      <c r="F6" s="14"/>
       <c r="G6" s="13"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="5"/>
-      <c r="B7" s="11"/>
+      <c r="A7" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="11" t="s">
+        <v>13</v>
+      </c>
       <c r="C7" s="12"/>
-      <c r="D7" s="12"/>
+      <c r="D7" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="E7" s="13"/>
+      <c r="F7" s="14"/>
       <c r="G7" s="13"/>
+      <c r="I7" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="J7" s="1" t="n">
+        <v>5000</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="15"/>
-      <c r="B8" s="16" t="s">
-        <v>9</v>
-      </c>
-      <c r="C8" s="17"/>
-      <c r="D8" s="17"/>
-      <c r="E8" s="18"/>
+      <c r="A8" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="C8" s="12"/>
+      <c r="D8" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" s="13"/>
       <c r="F8" s="14"/>
       <c r="G8" s="13"/>
+      <c r="I8" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="J8" s="1" t="n">
+        <v>2000</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="5"/>
-      <c r="B9" s="19"/>
-      <c r="C9" s="20"/>
-      <c r="D9" s="20"/>
-      <c r="E9" s="21"/>
+      <c r="A9" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="C9" s="12"/>
+      <c r="D9" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="E9" s="13"/>
       <c r="F9" s="14"/>
       <c r="G9" s="13"/>
     </row>
-    <row r="10" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="2"/>
-      <c r="B10" s="22" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="C10" s="12"/>
+      <c r="D10" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="E10" s="13"/>
+      <c r="F10" s="14"/>
+      <c r="G10" s="13"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="5" t="n">
         <v>10</v>
       </c>
-      <c r="C10" s="23"/>
-      <c r="D10" s="23"/>
-      <c r="E10" s="24" t="n">
-        <f aca="false">SUM(E2:E9)</f>
-        <v>650</v>
-      </c>
-      <c r="F10" s="25"/>
-      <c r="G10" s="21"/>
-    </row>
-    <row r="12" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E12" s="1" t="s">
+      <c r="B11" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="C11" s="12"/>
+      <c r="D11" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="E11" s="13" t="n">
+        <f aca="false">C11*D11</f>
+        <v>0</v>
+      </c>
+      <c r="F11" s="14"/>
+      <c r="G11" s="13"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="5" t="n">
         <v>11</v>
       </c>
-      <c r="F12" s="1" t="n">
-        <v>5000</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E13" s="1" t="s">
+      <c r="B12" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="C12" s="12"/>
+      <c r="D12" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="E12" s="13" t="n">
+        <f aca="false">C12*D12</f>
+        <v>0</v>
+      </c>
+      <c r="G12" s="13"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="5" t="n">
         <v>12</v>
       </c>
-      <c r="F13" s="1" t="n">
-        <v>2000</v>
-      </c>
-    </row>
-    <row r="1048556" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048557" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048558" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048559" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048560" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048561" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048562" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048563" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048564" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048565" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048566" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048567" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048568" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048569" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048570" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048571" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048572" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048573" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+      <c r="B13" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="C13" s="12"/>
+      <c r="D13" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="E13" s="13"/>
+      <c r="G13" s="13"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="C14" s="12"/>
+      <c r="D14" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" s="13"/>
+      <c r="G14" s="13"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="5" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="C15" s="12"/>
+      <c r="D15" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="E15" s="13"/>
+      <c r="G15" s="13"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="C16" s="12"/>
+      <c r="D16" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="E16" s="13"/>
+      <c r="G16" s="13"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="5" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="11" t="s">
+        <v>25</v>
+      </c>
+      <c r="C17" s="12"/>
+      <c r="D17" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" s="13"/>
+      <c r="G17" s="13"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="5" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="C18" s="12"/>
+      <c r="D18" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="E18" s="13"/>
+      <c r="G18" s="13"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="5" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="C19" s="12"/>
+      <c r="D19" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E19" s="13"/>
+      <c r="G19" s="13"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="5" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="C20" s="12"/>
+      <c r="D20" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" s="13"/>
+      <c r="G20" s="13"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="C21" s="12"/>
+      <c r="D21" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" s="13"/>
+      <c r="G21" s="13"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="5" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="C22" s="12"/>
+      <c r="D22" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E22" s="13"/>
+      <c r="G22" s="13"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="5" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="C23" s="12"/>
+      <c r="D23" s="12" t="n">
+        <v>6</v>
+      </c>
+      <c r="E23" s="13"/>
+      <c r="G23" s="13"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="5" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="C24" s="12"/>
+      <c r="D24" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E24" s="13"/>
+      <c r="G24" s="13"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="5" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="C25" s="12"/>
+      <c r="D25" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="E25" s="13"/>
+      <c r="G25" s="13"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="C26" s="12"/>
+      <c r="D26" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E26" s="13"/>
+      <c r="G26" s="13"/>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="5"/>
+      <c r="B27" s="11"/>
+      <c r="C27" s="12"/>
+      <c r="D27" s="12"/>
+      <c r="E27" s="13"/>
+      <c r="G27" s="13"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="5"/>
+      <c r="B28" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="C28" s="12" t="n">
+        <v>180</v>
+      </c>
+      <c r="D28" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E28" s="13"/>
+      <c r="G28" s="13"/>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="5"/>
+      <c r="B29" s="11"/>
+      <c r="C29" s="12"/>
+      <c r="D29" s="12"/>
+      <c r="E29" s="13"/>
+      <c r="G29" s="13"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="15"/>
+      <c r="B30" s="16" t="s">
+        <v>36</v>
+      </c>
+      <c r="C30" s="17"/>
+      <c r="D30" s="17"/>
+      <c r="E30" s="18"/>
+      <c r="F30" s="14"/>
+      <c r="G30" s="13"/>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="5"/>
+      <c r="B31" s="19"/>
+      <c r="C31" s="20"/>
+      <c r="D31" s="20"/>
+      <c r="E31" s="21"/>
+      <c r="F31" s="14"/>
+      <c r="G31" s="13"/>
+    </row>
+    <row r="32" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="2"/>
+      <c r="B32" s="22" t="s">
+        <v>37</v>
+      </c>
+      <c r="C32" s="23"/>
+      <c r="D32" s="23"/>
+      <c r="E32" s="24" t="n">
+        <f aca="false">SUM(E2:E31)</f>
+        <v>0</v>
+      </c>
+      <c r="F32" s="25"/>
+      <c r="G32" s="21"/>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E34" s="0"/>
+      <c r="F34" s="0"/>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E35" s="0"/>
+      <c r="F35" s="0"/>
+      <c r="G35" s="0"/>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F36" s="0"/>
+      <c r="G36" s="0"/>
+    </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>